<commit_message>
Add Census & Collections tab (1-month collection lag) to Refuge proforma
ADC -> patient days -> gross/net earned -> cash collected on a one-month lag,
with the recommended offer overlaid. Min cash $84.5K (Dec) under the 1-mo lag
vs $42.8K under the conservative 45-day-AR view.

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
+++ b/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer &amp; Affordability" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12-Mo P&amp;L (Operating Budget)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash-Flow Budget" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Census &amp; Collections" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,7 +52,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +128,7 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2480,6 +2487,591 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CENSUS -&gt; PATIENT DAYS -&gt; REVENUE -&gt; CASH (one-month collection lag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revenue is EARNED as patients are seen; cash is COLLECTED one month later (see patients in July, money lands in August). Expenses paid in-month (conservative: no AP lag credit). Recommended offer structure overlaid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>($/month)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Apr-27</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>May-27</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>Jun-27</t>
+        </is>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Average daily census (ADC)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total patient days</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>364.8</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>601.92</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>668.8</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>674.88</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>680.9599999999999</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>690.0799999999999</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>696.16</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>702.24</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>708.3199999999999</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>717.4400000000001</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>723.52</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>729.5999999999999</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>7958.720000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gross revenue (earned)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>67592.10049535999</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>111526.965817344</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>123918.85090816</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>125045.385916416</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>126171.920924672</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>127861.723437056</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>128988.258445312</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>130114.793453568</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>131241.328461824</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>132931.130974208</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>134057.665982464</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>135184.20099072</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>1474634.325807104</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>NET REVENUE (earned)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>66138.87033470976</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>109129.1360522711</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>121254.5956136346</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>122356.9101192131</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>123459.2246247915</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>125112.6963831593</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>126215.0108887378</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>127317.3253943163</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>128419.6398998948</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>130073.1116582626</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>131175.426163841</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>132277.7406694195</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>1442929.687802251</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Cash COLLECTED (prior month's net)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>66138.87033470976</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>109129.1360522711</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>121254.5956136346</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>122356.9101192131</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>123459.2246247915</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>125112.6963831593</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>126215.0108887378</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>127317.3253943163</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>128419.6398998948</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>130073.1116582626</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>131175.426163841</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>1310651.947132832</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Operating expenses (cash, in-month)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>-55099.15800281227</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>-71748.72559422356</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>-86594.37713710028</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>-94671.8649864527</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>-94806.68936913845</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>-104921.9676098338</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>-105056.7919925195</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>-105191.6163752053</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>-105326.440757891</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>-105528.6773319197</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>-105663.5017146054</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>-105798.3260972912</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>-1140408.136968993</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Net operating cash</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>-55099.15800281227</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>-5609.855259513803</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>22534.75891517082</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>26582.73062718187</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>27550.22075007462</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>18537.25701495777</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>20055.90439063976</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>21023.3945135325</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>21990.88463642525</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>22890.9625679751</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>24409.60994365711</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>25377.10006654984</v>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>170243.8101638386</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Seller payments (down excl.)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>-100000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Refi principal+interest (M7+)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>-3942.783457976496</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>-23656.70074785898</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ENDING CASH (1-mo lag view)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>94900.84199718773</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>89290.98673767393</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>86825.74565284477</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>88408.47628002665</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>90958.69703010126</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>84495.95404505901</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>100609.0749777223</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>117689.6860332783</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>135737.787211727</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>154685.9663217257</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>175152.7928074063</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>196587.1094159796</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Min cash $84,496 (Dec-26)  |  End Jun-27 $196,587  |  vs 45-day-AR view min $42,750 - the one-month lag is the better case; the 45-day view is the conservative floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Six-month picture: net revenue earned Jul-Dec ~$667K; collected by Dec 31 ~$542K (December's revenue lands in January). EBITDA positive every month from M1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Operating-cost interview refinements + full sensitivity grid
Interview-locked cost refinements: G&A -$2,004/mo (rent $2,000, cut CC fees),
health 90-day waiting period, med director contracted; salaries firm/timing
census-tracked; owner deferral (~$12K/mo M1-6) as downside lever.

refuge_sensitivity.py: census-capture x payroll grid with 1-mo-lag and 45-day-AR
cash paths, breakeven ADC (17.9; 19.5 at +10% payroll), max-seller-monthly solver,
$25K floor verdicts. Cliff: safe to 82% capture (90% at +10% payroll).
Workbook: new Sensitivity tab; refined base min cash $97K (lag-1) / $61K (AR45).

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
+++ b/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12-Mo P&amp;L (Operating Budget)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash-Flow Budget" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Census &amp; Collections" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -111,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +130,7 @@
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3072,6 +3074,376 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SENSITIVITY - census capture x payroll inflation (interview-locked axes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cost refinements applied to ALL cases: G&amp;A -$2,004/mo (rent $2,000; credit-card fees cut); health insurance 90-day waiting period; med director contracted (not inflated). Floor: &gt;=$25K safe | &lt;$25K flag | &lt;$0 FAIL. Offer overlay: $100K down + $25K x4 (M3-6) + Jan balloon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>6-mo EBITDA</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Min cash (1-mo lag)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Trough mo</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Min cash (45-day AR)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Base (100% capture)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>182082.6504282183</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>97148.98673767391</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>60717.56239189742</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Census 85%</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>94210.36001648555</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>37864.56809080014</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>4446.684479689873</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Census 70%</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>6338.069604752796</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>-108064.9396431718</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>-134132.717135684</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Census 55%</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>-81534.22080697989</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>-278189.9641727477</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>-295244.7666958674</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Payroll +10%</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>147963.1498501349</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>72850.4534669756</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>31104.35587495734</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Payroll +15%</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>130903.3995610933</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>55790.70317793399</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>14044.60558591575</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Census 85% + payroll +10%</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>60588.74524036469</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>-17725.75802035446</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>-53114.88296519467</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>COMBINED: census 70% + pay +10%</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>-26785.65936940556</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>-186774.4282728553</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>-212523.9124518816</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Combined + owner deferral</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>45214.34063059444</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>-114774.4282728552</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>-141661.087653699</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>WHERE THE CLIFF IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Safe ($25K floor) down to 82% census capture (steady ADC ~18.7). Never-negative down to 80% (ADC ~18.1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - If payroll runs +10%, the safe threshold rises to 90% capture; owner deferral buys it back to ~80%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Breakeven ADC (steady state): 17.9 patients; at payroll +10%: 19.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Below ~80% capture the BUSINESS is EBITDA-negative at steady state - no offer structure fixes that;</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - the mitigation is the census ramp itself (marketing, referral push), not deal terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>MAX AFFORDABLE SELLER MONTHLY (M3-6, after $100K down; $25K floor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Base (100%): $45,492/mo  (offer's $25K has ~$20K headroom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Census 85%: $28,216/mo  (offer's $25K still fits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Census 70%: $0/mo  (payments would need pause/cure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Interview-locked mitigations: hires track census (natural hedge); owner salary deferral ~$12K/mo available M1-6; LOI cure/pause language on monthlies recommended for the &lt;85% case.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Project cash flow under Jorge/Dennis 7/5 counter (125K + 25K Aug-Dec + Jan balloon)
Counter as-is: min cash $47.1K expected / $10.7K on 45-day AR (below $25K floor);
fails at 85% census. One-month tweak (Sep start, 4 pmts, balloon ~$285.5K): $72.1K /
$35.7K - safe both views, survives payroll +10%, deferral rescues combined case.
New 'Seller Counter (Jul 5)' workbook tab with both paths + verdict.

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
+++ b/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12-Mo P&amp;L (Operating Budget)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash-Flow Budget" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Census &amp; Collections" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seller Counter (Jul 5)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3074,6 +3075,421 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SELLER COUNTER 7/5: $125K down + $25K/mo AUG-DEC (5 pmts) + Jan balloon @6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Jorge/Dennis counter accepts our price and hybrid structure but starts monthlies in August (inside the collections-lag window) and adds a 5th payment. Seller receives $250K (50%) pre-balloon. Balloon ~$260,000 (incl. ~$10,000 interest), refi-funded in January.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>($/month)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Apr-27</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>May-27</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>Jun-27</t>
+        </is>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cash collected (1-mo lag)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>66138.87033470976</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>109129.1360522711</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>121254.5956136346</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>122356.9101192131</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>123459.2246247915</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>125112.6963831593</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>126215.0108887378</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>127317.3253943163</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>128419.6398998948</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>130073.1116582626</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>131175.426163841</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>1310651.947132832</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Operating expenses (refined costs)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>-51445.15800281227</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-67544.72559422358</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-81840.37713710027</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-91017.8649864527</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-91702.68936913846</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>-101817.9676098338</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-102502.7919925195</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>-102637.6163752053</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>-103322.440757891</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>-103524.6773319197</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>-103659.5017146054</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>-103794.3260972912</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>-1104810.136968993</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Seller payments - COUNTER (Aug start)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>-125000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ENDING CASH - counter as-is</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>73554.84199718773</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>47148.98673767391</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>49437.74565284475</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>54674.47628002662</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>60328.69703010122</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>56969.95404505901</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>76286.28831819232</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>96570.11271421838</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>117271.4272331372</v>
+      </c>
+      <c r="K8" s="14" t="n">
+        <v>138872.8196836058</v>
+      </c>
+      <c r="L8" s="14" t="n">
+        <v>161992.8595097565</v>
+      </c>
+      <c r="M8" s="14" t="n">
+        <v>186080.3894587998</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Seller payments - TWEAK (Sep start)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>-100000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ENDING CASH - with Sep-start tweak</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>73554.84199718773</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>72148.98673767391</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>74437.74565284475</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>79674.47628002662</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>85328.69703010122</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>81969.95404505901</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>100963.2650951292</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>120924.0662680921</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>141302.3575639478</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>162580.7267913533</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>185377.7433944408</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>209142.2501204211</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Counter as-is: min cash $47,149 (Aug) expected-case; $10,718 (Sep) on the conservative 45-day view - passes the $25K floor only on expected collections; FAILS at 85% census (-$12K).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - One-month tweak (first payment September, 4 pmts, balloon $285,500): min cash $72,149 expected / ~$35.7K conservative - safe on BOTH views, survives payroll +10%, and the combined downside is rescued by owner deferral. Seller still gets $225K (45%) by December and full payout in January.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Recommendation: accept the counter with the single September-start adjustment (or accept as-is only with a 30-day cure/grace clause on the monthlies).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3438,7 +3854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Model September $500K/6%/36mo full refinance scenario
Close on counter front end (125K down + 25K Aug), refi entire 500K in Sept:
sellers paid in full (~$355.5K) end-Sept, ~$144.5K surplus to working capital,
$15,211/mo x36 from October. Min cash $47.1K expected / ~$14K 45-day (Aug pinch);
cash builds to $313K by June; all 12-mo stress cases positive. Trade-off: steady
DSCR 1.87x base but 0.73x at 85% census - note not self-supporting in slow-ramp
world. New 'Sep Refi $500K' workbook tab.

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
+++ b/financial_models/output/Azalea_Refuge_12mo_Proforma.xlsx
@@ -13,8 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash-Flow Budget" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Census &amp; Collections" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seller Counter (Jul 5)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep Refi $500K" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SBA Scenario" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3490,6 +3491,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SEPTEMBER REFI: $500,000 @ 6% / 36 months - sellers paid in full end-September</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Close on the counter's front end ($125K down Jul + $25K Aug), then refinance the entire $500K in September: pay the sellers off (~$355,500 incl. ~$5,500 interest) and keep the ~$144,500 surplus as working capital. No January balloon. Loan service $15,211/mo ($182,532/yr) starting October for 36 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>($/month)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Apr-27</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>May-27</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>Jun-27</t>
+        </is>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cash collected (1-mo lag)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>66138.87033470976</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>109129.1360522711</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>121254.5956136346</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>122356.9101192131</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>123459.2246247915</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>125112.6963831593</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>126215.0108887378</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>127317.3253943163</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>128419.6398998948</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>130073.1116582626</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>131175.426163841</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>1310651.947132832</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Operating expenses (refined costs)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>-51445.15800281227</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-67544.72559422358</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-81840.37713710027</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-91017.8649864527</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-91702.68936913846</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>-101817.9676098338</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-102502.7919925195</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>-102637.6163752053</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>-103322.440757891</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>-103524.6773319197</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>-103659.5017146054</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>-103794.3260972912</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>-1104810.136968993</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Acquisition / loan cash flows</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>-125000</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>144500</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>-15210.96872577785</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>-142398.7185320007</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ENDING CASH</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>73554.84199718773</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>47148.98673767391</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>218937.7456528448</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>233963.5075542488</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>249406.7595785456</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>255837.0478677256</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>263235.9835325875</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>271602.4093203421</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>280386.3252309895</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>290070.3190731868</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>301272.960291066</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>313443.091631838</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Min cash $47,149 (Aug) expected-case; ~$14,000 (Aug) on the conservative 45-day view - August is still the pinch (fix: ask to skip the August $25K since they're paid in full in September; that lifts the trough to ~$72K / ~$39K).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - After the September surplus lands, cash jumps to ~$219K and climbs to ~$313K by June - every 12-month stress case stays positive (worst: ~$33K at census 85% + payroll +10%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - THE TRADE-OFF: $15,211/mo for 36 months is heavy amortization. Steady-state DSCR is 1.87x in the base case but falls BELOW 1.0x at 85% census (0.73x) - in a slow-ramp world the note is not self-supporting from operations and the ~$144K surplus becomes the shock absorber for years 2-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Versus the January-balloon plan: sellers paid 4 months earlier (a strong negotiating chip), no balloon/refi-timing risk, cheaper rate (6% vs ~9%) - in exchange for locked-in heavy payments for 3 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - If the SBA $450K also lands, combined service is ~$242K/yr vs steady EBITDA ~$342K/yr (1.41x) - workable but disclose the piggyback to the SBA lender.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3854,7 +4195,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>